<commit_message>
joints: a Voronoi cell wall shorter than a tenth of the block size is dropped as a sliver; mesh: a line no longer than the snap tolerance is refused with a plain message
The tutorial's Voronoi model carried a 6.7 cm cell wall that the mesher's
end-snapping folded to nothing, and the failure surfaced as a ZeroDivisionError
downstream. The generator now floors wall length at a tenth of the block size
(the model goes from 59 to 51 lines and meshes at 1,303 nodes), and the mesher
names a sub-tolerance line and what to do about it instead of failing on the
arithmetic.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_rock_voronoi.xlsx
+++ b/docs/tutorials/files/xslope_rock_voronoi.xlsx
@@ -4994,16 +4994,16 @@
         </is>
       </c>
       <c r="C5" s="3">
-        <v>20.4450364601</v>
+        <v>20.3780073462</v>
       </c>
       <c r="D5" s="3">
-        <v>0.8368693944</v>
+        <v>0.8332298825</v>
       </c>
       <c r="E5" s="3">
-        <v>20.3780073462</v>
+        <v>19.6154175935</v>
       </c>
       <c r="F5" s="3">
-        <v>0.8332298825</v>
+        <v>1.5831123016</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3">
@@ -5027,16 +5027,16 @@
         </is>
       </c>
       <c r="C6" s="3">
-        <v>20.3780073462</v>
+        <v>19.056395489</v>
       </c>
       <c r="D6" s="3">
-        <v>0.8332298825</v>
+        <v>3.2420661099</v>
       </c>
       <c r="E6" s="3">
-        <v>19.6154175935</v>
+        <v>18.1740303359</v>
       </c>
       <c r="F6" s="3">
-        <v>1.5831123016</v>
+        <v>3.4451336165</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3">
@@ -5060,16 +5060,16 @@
         </is>
       </c>
       <c r="C7" s="3">
-        <v>19.056395489</v>
+        <v>19.6154175935</v>
       </c>
       <c r="D7" s="3">
-        <v>3.2420661099</v>
+        <v>1.5831123016</v>
       </c>
       <c r="E7" s="3">
-        <v>18.1740303359</v>
+        <v>18.8083707781</v>
       </c>
       <c r="F7" s="3">
-        <v>3.4451336165</v>
+        <v>1.2238858369</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3">
@@ -5093,16 +5093,16 @@
         </is>
       </c>
       <c r="C8" s="3">
-        <v>19.6154175935</v>
+        <v>18.1788913758</v>
       </c>
       <c r="D8" s="3">
-        <v>1.5831123016</v>
+        <v>1.5873159393</v>
       </c>
       <c r="E8" s="3">
-        <v>18.8083707781</v>
+        <v>17.2037996937</v>
       </c>
       <c r="F8" s="3">
-        <v>1.2238858369</v>
+        <v>2.8974761555</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3">
@@ -5126,10 +5126,10 @@
         </is>
       </c>
       <c r="C9" s="3">
-        <v>18.1788913758</v>
+        <v>18.1740303359</v>
       </c>
       <c r="D9" s="3">
-        <v>1.5873159393</v>
+        <v>3.4451336165</v>
       </c>
       <c r="E9" s="3">
         <v>17.2037996937</v>
@@ -5165,10 +5165,10 @@
         <v>3.4451336165</v>
       </c>
       <c r="E10" s="3">
-        <v>17.2037996937</v>
+        <v>18.3323587154</v>
       </c>
       <c r="F10" s="3">
-        <v>2.8974761555</v>
+        <v>4.4961345883</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3">
@@ -5192,16 +5192,16 @@
         </is>
       </c>
       <c r="C11" s="3">
-        <v>18.1740303359</v>
+        <v>16.6668237583</v>
       </c>
       <c r="D11" s="3">
-        <v>3.4451336165</v>
+        <v>2.4603085853</v>
       </c>
       <c r="E11" s="3">
-        <v>18.3323587154</v>
+        <v>17.0101565955</v>
       </c>
       <c r="F11" s="3">
-        <v>4.4961345883</v>
+        <v>2.9371281221</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3">
@@ -5225,16 +5225,16 @@
         </is>
       </c>
       <c r="C12" s="3">
-        <v>16.6668237583</v>
+        <v>20.3780073462</v>
       </c>
       <c r="D12" s="3">
-        <v>2.4603085853</v>
+        <v>0.8332298825</v>
       </c>
       <c r="E12" s="3">
-        <v>17.0101565955</v>
+        <v>20.4021028897</v>
       </c>
       <c r="F12" s="3">
-        <v>2.9371281221</v>
+        <v>0.3037441732</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3">
@@ -5258,16 +5258,16 @@
         </is>
       </c>
       <c r="C13" s="3">
+        <v>15.8942747876</v>
+      </c>
+      <c r="D13" s="3">
+        <v>4.3062658691</v>
+      </c>
+      <c r="E13" s="3">
         <v>17.0101565955</v>
       </c>
-      <c r="D13" s="3">
+      <c r="F13" s="3">
         <v>2.9371281221</v>
-      </c>
-      <c r="E13" s="3">
-        <v>17.2037996937</v>
-      </c>
-      <c r="F13" s="3">
-        <v>2.8974761555</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="3">
@@ -5291,16 +5291,16 @@
         </is>
       </c>
       <c r="C14" s="3">
-        <v>20.3780073462</v>
+        <v>15.8942747876</v>
       </c>
       <c r="D14" s="3">
-        <v>0.8332298825</v>
+        <v>4.3062658691</v>
       </c>
       <c r="E14" s="3">
-        <v>20.4021028897</v>
+        <v>15.1907076895</v>
       </c>
       <c r="F14" s="3">
-        <v>0.3037441732</v>
+        <v>3.3125445949</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3">
@@ -5330,10 +5330,10 @@
         <v>4.3062658691</v>
       </c>
       <c r="E15" s="3">
-        <v>17.0101565955</v>
+        <v>15.7740495512</v>
       </c>
       <c r="F15" s="3">
-        <v>2.9371281221</v>
+        <v>4.8379423909</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3">
@@ -5357,16 +5357,16 @@
         </is>
       </c>
       <c r="C16" s="3">
-        <v>15.8942747876</v>
+        <v>17.9404625039</v>
       </c>
       <c r="D16" s="3">
-        <v>4.3062658691</v>
+        <v>5.1749187379</v>
       </c>
       <c r="E16" s="3">
-        <v>15.1907076895</v>
+        <v>15.80159514</v>
       </c>
       <c r="F16" s="3">
-        <v>3.3125445949</v>
+        <v>4.8848227473</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3">
@@ -5390,16 +5390,16 @@
         </is>
       </c>
       <c r="C17" s="3">
-        <v>15.8942747876</v>
+        <v>13.4550465205</v>
       </c>
       <c r="D17" s="3">
-        <v>4.3062658691</v>
+        <v>4.3146290381</v>
       </c>
       <c r="E17" s="3">
-        <v>15.7740495512</v>
+        <v>13.5428139331</v>
       </c>
       <c r="F17" s="3">
-        <v>4.8379423909</v>
+        <v>4.8193934506</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="3">
@@ -5423,16 +5423,16 @@
         </is>
       </c>
       <c r="C18" s="3">
-        <v>17.9404625039</v>
+        <v>15.7740495512</v>
       </c>
       <c r="D18" s="3">
-        <v>5.1749187379</v>
+        <v>4.8379423909</v>
       </c>
       <c r="E18" s="3">
-        <v>15.80159514</v>
+        <v>13.5428139331</v>
       </c>
       <c r="F18" s="3">
-        <v>4.8848227473</v>
+        <v>4.8193934506</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3">
@@ -5456,16 +5456,16 @@
         </is>
       </c>
       <c r="C19" s="3">
-        <v>15.7740495512</v>
+        <v>12.7224468968</v>
       </c>
       <c r="D19" s="3">
-        <v>4.8379423909</v>
+        <v>5.1077385569</v>
       </c>
       <c r="E19" s="3">
-        <v>15.80159514</v>
+        <v>13.3593466902</v>
       </c>
       <c r="F19" s="3">
-        <v>4.8848227473</v>
+        <v>4.9737643734</v>
       </c>
       <c r="G19" s="3"/>
       <c r="H19" s="3">
@@ -5489,16 +5489,16 @@
         </is>
       </c>
       <c r="C20" s="3">
-        <v>13.4550465205</v>
+        <v>12.7224468968</v>
       </c>
       <c r="D20" s="3">
-        <v>4.3146290381</v>
+        <v>5.1077385569</v>
       </c>
       <c r="E20" s="3">
-        <v>13.5428139331</v>
+        <v>12.3909149015</v>
       </c>
       <c r="F20" s="3">
-        <v>4.8193934506</v>
+        <v>4.9290057148</v>
       </c>
       <c r="G20" s="3"/>
       <c r="H20" s="3">
@@ -5522,16 +5522,16 @@
         </is>
       </c>
       <c r="C21" s="3">
-        <v>15.7740495512</v>
+        <v>13.5428139331</v>
       </c>
       <c r="D21" s="3">
-        <v>4.8379423909</v>
+        <v>4.8193934506</v>
       </c>
       <c r="E21" s="3">
-        <v>13.5428139331</v>
+        <v>13.3593466902</v>
       </c>
       <c r="F21" s="3">
-        <v>4.8193934506</v>
+        <v>4.9737643734</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3">
@@ -5555,16 +5555,16 @@
         </is>
       </c>
       <c r="C22" s="3">
-        <v>12.7224468968</v>
+        <v>9.9933493828</v>
       </c>
       <c r="D22" s="3">
-        <v>5.1077385569</v>
+        <v>6.3663863134</v>
       </c>
       <c r="E22" s="3">
-        <v>13.3593466902</v>
+        <v>9.0</v>
       </c>
       <c r="F22" s="3">
-        <v>4.9737643734</v>
+        <v>7.1796820917</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3">
@@ -5594,10 +5594,10 @@
         <v>5.1077385569</v>
       </c>
       <c r="E23" s="3">
-        <v>12.3909149015</v>
+        <v>11.4501932026</v>
       </c>
       <c r="F23" s="3">
-        <v>4.9290057148</v>
+        <v>7.0521399654</v>
       </c>
       <c r="G23" s="3"/>
       <c r="H23" s="3">
@@ -5621,16 +5621,16 @@
         </is>
       </c>
       <c r="C24" s="3">
-        <v>13.5428139331</v>
+        <v>9.9933493828</v>
       </c>
       <c r="D24" s="3">
-        <v>4.8193934506</v>
+        <v>6.3663863134</v>
       </c>
       <c r="E24" s="3">
-        <v>13.3593466902</v>
+        <v>10.8673381917</v>
       </c>
       <c r="F24" s="3">
-        <v>4.9737643734</v>
+        <v>6.975070257</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3">
@@ -5654,16 +5654,16 @@
         </is>
       </c>
       <c r="C25" s="3">
-        <v>9.9933493828</v>
+        <v>11.4501932026</v>
       </c>
       <c r="D25" s="3">
-        <v>6.3663863134</v>
+        <v>7.0521399654</v>
       </c>
       <c r="E25" s="3">
-        <v>9.0</v>
+        <v>10.8673381917</v>
       </c>
       <c r="F25" s="3">
-        <v>7.1796820917</v>
+        <v>6.975070257</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3">
@@ -5687,16 +5687,16 @@
         </is>
       </c>
       <c r="C26" s="3">
-        <v>9.9933493828</v>
+        <v>9.0</v>
       </c>
       <c r="D26" s="3">
-        <v>6.3663863134</v>
+        <v>8.5928442153</v>
       </c>
       <c r="E26" s="3">
-        <v>9.9807034801</v>
+        <v>9.9349667823</v>
       </c>
       <c r="F26" s="3">
-        <v>6.3205419277</v>
+        <v>9.3471048166</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3">
@@ -5720,16 +5720,16 @@
         </is>
       </c>
       <c r="C27" s="3">
-        <v>12.7224468968</v>
+        <v>10.8673381917</v>
       </c>
       <c r="D27" s="3">
-        <v>5.1077385569</v>
+        <v>6.975070257</v>
       </c>
       <c r="E27" s="3">
-        <v>11.4501932026</v>
+        <v>9.9349667823</v>
       </c>
       <c r="F27" s="3">
-        <v>7.0521399654</v>
+        <v>9.3471048166</v>
       </c>
       <c r="G27" s="3"/>
       <c r="H27" s="3">
@@ -5753,16 +5753,16 @@
         </is>
       </c>
       <c r="C28" s="3">
-        <v>9.9933493828</v>
+        <v>9.0270277098</v>
       </c>
       <c r="D28" s="3">
-        <v>6.3663863134</v>
+        <v>10.9146343248</v>
       </c>
       <c r="E28" s="3">
-        <v>10.8673381917</v>
+        <v>9.94722374</v>
       </c>
       <c r="F28" s="3">
-        <v>6.975070257</v>
+        <v>9.383846683</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3">
@@ -5786,16 +5786,16 @@
         </is>
       </c>
       <c r="C29" s="3">
-        <v>11.4501932026</v>
+        <v>12.6531707391</v>
       </c>
       <c r="D29" s="3">
-        <v>7.0521399654</v>
+        <v>12.0</v>
       </c>
       <c r="E29" s="3">
-        <v>10.8673381917</v>
+        <v>12.1925700451</v>
       </c>
       <c r="F29" s="3">
-        <v>6.975070257</v>
+        <v>10.582869313</v>
       </c>
       <c r="G29" s="3"/>
       <c r="H29" s="3">
@@ -5819,16 +5819,16 @@
         </is>
       </c>
       <c r="C30" s="3">
-        <v>9.0</v>
+        <v>12.1925700451</v>
       </c>
       <c r="D30" s="3">
-        <v>8.5928442153</v>
+        <v>10.582869313</v>
       </c>
       <c r="E30" s="3">
-        <v>9.9349667823</v>
+        <v>10.4484473738</v>
       </c>
       <c r="F30" s="3">
-        <v>9.3471048166</v>
+        <v>11.7015984609</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3">
@@ -5852,16 +5852,16 @@
         </is>
       </c>
       <c r="C31" s="3">
-        <v>10.8673381917</v>
+        <v>10.4484473738</v>
       </c>
       <c r="D31" s="3">
-        <v>6.975070257</v>
+        <v>11.7015984609</v>
       </c>
       <c r="E31" s="3">
-        <v>9.9349667823</v>
+        <v>10.5081599955</v>
       </c>
       <c r="F31" s="3">
-        <v>9.3471048166</v>
+        <v>12.0</v>
       </c>
       <c r="G31" s="3"/>
       <c r="H31" s="3">
@@ -5891,10 +5891,10 @@
         <v>10.9146343248</v>
       </c>
       <c r="E32" s="3">
-        <v>9.0</v>
+        <v>10.4484473738</v>
       </c>
       <c r="F32" s="3">
-        <v>10.9234428093</v>
+        <v>11.7015984609</v>
       </c>
       <c r="G32" s="3"/>
       <c r="H32" s="3">
@@ -5918,16 +5918,16 @@
         </is>
       </c>
       <c r="C33" s="3">
-        <v>9.0270277098</v>
+        <v>16.7569157788</v>
       </c>
       <c r="D33" s="3">
-        <v>10.9146343248</v>
+        <v>7.224881799</v>
       </c>
       <c r="E33" s="3">
-        <v>9.94722374</v>
+        <v>15.9343070195</v>
       </c>
       <c r="F33" s="3">
-        <v>9.383846683</v>
+        <v>7.0542242354</v>
       </c>
       <c r="G33" s="3"/>
       <c r="H33" s="3">
@@ -5951,16 +5951,16 @@
         </is>
       </c>
       <c r="C34" s="3">
-        <v>9.94722374</v>
+        <v>15.881093899</v>
       </c>
       <c r="D34" s="3">
-        <v>9.383846683</v>
+        <v>8.7418497931</v>
       </c>
       <c r="E34" s="3">
-        <v>9.9349667823</v>
+        <v>15.9343070195</v>
       </c>
       <c r="F34" s="3">
-        <v>9.3471048166</v>
+        <v>7.0542242354</v>
       </c>
       <c r="G34" s="3"/>
       <c r="H34" s="3">
@@ -5984,16 +5984,16 @@
         </is>
       </c>
       <c r="C35" s="3">
-        <v>12.6531707391</v>
+        <v>15.80159514</v>
       </c>
       <c r="D35" s="3">
-        <v>12.0</v>
+        <v>4.8848227473</v>
       </c>
       <c r="E35" s="3">
-        <v>12.1925700451</v>
+        <v>15.9140073835</v>
       </c>
       <c r="F35" s="3">
-        <v>10.582869313</v>
+        <v>7.0339111337</v>
       </c>
       <c r="G35" s="3"/>
       <c r="H35" s="3">
@@ -6017,16 +6017,16 @@
         </is>
       </c>
       <c r="C36" s="3">
-        <v>12.1925700451</v>
+        <v>13.3593466902</v>
       </c>
       <c r="D36" s="3">
-        <v>10.582869313</v>
+        <v>4.9737643734</v>
       </c>
       <c r="E36" s="3">
-        <v>10.4484473738</v>
+        <v>13.7481247121</v>
       </c>
       <c r="F36" s="3">
-        <v>11.7015984609</v>
+        <v>7.1049048955</v>
       </c>
       <c r="G36" s="3"/>
       <c r="H36" s="3">
@@ -6050,16 +6050,16 @@
         </is>
       </c>
       <c r="C37" s="3">
-        <v>10.4484473738</v>
+        <v>15.9140073835</v>
       </c>
       <c r="D37" s="3">
-        <v>11.7015984609</v>
+        <v>7.0339111337</v>
       </c>
       <c r="E37" s="3">
-        <v>10.5081599955</v>
+        <v>14.3608123661</v>
       </c>
       <c r="F37" s="3">
-        <v>12.0</v>
+        <v>7.4155502673</v>
       </c>
       <c r="G37" s="3"/>
       <c r="H37" s="3">
@@ -6083,16 +6083,16 @@
         </is>
       </c>
       <c r="C38" s="3">
-        <v>9.0270277098</v>
+        <v>13.7481247121</v>
       </c>
       <c r="D38" s="3">
-        <v>10.9146343248</v>
+        <v>7.1049048955</v>
       </c>
       <c r="E38" s="3">
-        <v>10.4484473738</v>
+        <v>14.3608123661</v>
       </c>
       <c r="F38" s="3">
-        <v>11.7015984609</v>
+        <v>7.4155502673</v>
       </c>
       <c r="G38" s="3"/>
       <c r="H38" s="3">
@@ -6116,16 +6116,16 @@
         </is>
       </c>
       <c r="C39" s="3">
-        <v>16.7569157788</v>
+        <v>11.4501932026</v>
       </c>
       <c r="D39" s="3">
-        <v>7.224881799</v>
+        <v>7.0521399654</v>
       </c>
       <c r="E39" s="3">
-        <v>15.9343070195</v>
+        <v>12.0382492411</v>
       </c>
       <c r="F39" s="3">
-        <v>7.0542242354</v>
+        <v>7.5687085359</v>
       </c>
       <c r="G39" s="3"/>
       <c r="H39" s="3">
@@ -6149,16 +6149,16 @@
         </is>
       </c>
       <c r="C40" s="3">
-        <v>15.881093899</v>
+        <v>13.7481247121</v>
       </c>
       <c r="D40" s="3">
-        <v>8.7418497931</v>
+        <v>7.1049048955</v>
       </c>
       <c r="E40" s="3">
-        <v>15.9343070195</v>
+        <v>12.0382492411</v>
       </c>
       <c r="F40" s="3">
-        <v>7.0542242354</v>
+        <v>7.5687085359</v>
       </c>
       <c r="G40" s="3"/>
       <c r="H40" s="3">
@@ -6182,16 +6182,16 @@
         </is>
       </c>
       <c r="C41" s="3">
-        <v>15.80159514</v>
+        <v>12.2927613852</v>
       </c>
       <c r="D41" s="3">
-        <v>4.8848227473</v>
+        <v>8.8982603035</v>
       </c>
       <c r="E41" s="3">
-        <v>15.9140073835</v>
+        <v>14.0108561039</v>
       </c>
       <c r="F41" s="3">
-        <v>7.0339111337</v>
+        <v>8.724001641</v>
       </c>
       <c r="G41" s="3"/>
       <c r="H41" s="3">
@@ -6215,16 +6215,16 @@
         </is>
       </c>
       <c r="C42" s="3">
-        <v>15.9343070195</v>
+        <v>12.2927613852</v>
       </c>
       <c r="D42" s="3">
-        <v>7.0542242354</v>
+        <v>8.8982603035</v>
       </c>
       <c r="E42" s="3">
-        <v>15.9140073835</v>
+        <v>11.9559488087</v>
       </c>
       <c r="F42" s="3">
-        <v>7.0339111337</v>
+        <v>9.8116238502</v>
       </c>
       <c r="G42" s="3"/>
       <c r="H42" s="3">
@@ -6248,16 +6248,16 @@
         </is>
       </c>
       <c r="C43" s="3">
-        <v>13.3593466902</v>
+        <v>11.9559488087</v>
       </c>
       <c r="D43" s="3">
-        <v>4.9737643734</v>
+        <v>9.8116238502</v>
       </c>
       <c r="E43" s="3">
-        <v>13.7481247121</v>
+        <v>12.2185604292</v>
       </c>
       <c r="F43" s="3">
-        <v>7.1049048955</v>
+        <v>10.4839102174</v>
       </c>
       <c r="G43" s="3"/>
       <c r="H43" s="3">
@@ -6281,16 +6281,16 @@
         </is>
       </c>
       <c r="C44" s="3">
-        <v>15.9140073835</v>
+        <v>12.2185604292</v>
       </c>
       <c r="D44" s="3">
-        <v>7.0339111337</v>
+        <v>10.4839102174</v>
       </c>
       <c r="E44" s="3">
-        <v>14.3608123661</v>
+        <v>13.9155797828</v>
       </c>
       <c r="F44" s="3">
-        <v>7.4155502673</v>
+        <v>10.3899370543</v>
       </c>
       <c r="G44" s="3"/>
       <c r="H44" s="3">
@@ -6314,16 +6314,16 @@
         </is>
       </c>
       <c r="C45" s="3">
-        <v>13.7481247121</v>
+        <v>13.9155797828</v>
       </c>
       <c r="D45" s="3">
-        <v>7.1049048955</v>
+        <v>10.3899370543</v>
       </c>
       <c r="E45" s="3">
-        <v>14.3608123661</v>
+        <v>14.1339424409</v>
       </c>
       <c r="F45" s="3">
-        <v>7.4155502673</v>
+        <v>10.2888438165</v>
       </c>
       <c r="G45" s="3"/>
       <c r="H45" s="3">
@@ -6347,16 +6347,16 @@
         </is>
       </c>
       <c r="C46" s="3">
-        <v>11.4501932026</v>
+        <v>14.1339424409</v>
       </c>
       <c r="D46" s="3">
-        <v>7.0521399654</v>
+        <v>10.2888438165</v>
       </c>
       <c r="E46" s="3">
-        <v>12.0382492411</v>
+        <v>14.421771329</v>
       </c>
       <c r="F46" s="3">
-        <v>7.5687085359</v>
+        <v>9.3533122858</v>
       </c>
       <c r="G46" s="3"/>
       <c r="H46" s="3">
@@ -6380,16 +6380,16 @@
         </is>
       </c>
       <c r="C47" s="3">
-        <v>13.7481247121</v>
+        <v>14.421771329</v>
       </c>
       <c r="D47" s="3">
-        <v>7.1049048955</v>
+        <v>9.3533122858</v>
       </c>
       <c r="E47" s="3">
-        <v>12.0382492411</v>
+        <v>14.0108561039</v>
       </c>
       <c r="F47" s="3">
-        <v>7.5687085359</v>
+        <v>8.724001641</v>
       </c>
       <c r="G47" s="3"/>
       <c r="H47" s="3">
@@ -6413,10 +6413,10 @@
         </is>
       </c>
       <c r="C48" s="3">
-        <v>12.2927613852</v>
+        <v>14.3608123661</v>
       </c>
       <c r="D48" s="3">
-        <v>8.8982603035</v>
+        <v>7.4155502673</v>
       </c>
       <c r="E48" s="3">
         <v>14.0108561039</v>
@@ -6446,16 +6446,16 @@
         </is>
       </c>
       <c r="C49" s="3">
+        <v>12.0382492411</v>
+      </c>
+      <c r="D49" s="3">
+        <v>7.5687085359</v>
+      </c>
+      <c r="E49" s="3">
         <v>12.2927613852</v>
       </c>
-      <c r="D49" s="3">
+      <c r="F49" s="3">
         <v>8.8982603035</v>
-      </c>
-      <c r="E49" s="3">
-        <v>11.9559488087</v>
-      </c>
-      <c r="F49" s="3">
-        <v>9.8116238502</v>
       </c>
       <c r="G49" s="3"/>
       <c r="H49" s="3">
@@ -6479,16 +6479,16 @@
         </is>
       </c>
       <c r="C50" s="3">
+        <v>9.94722374</v>
+      </c>
+      <c r="D50" s="3">
+        <v>9.383846683</v>
+      </c>
+      <c r="E50" s="3">
         <v>11.9559488087</v>
       </c>
-      <c r="D50" s="3">
+      <c r="F50" s="3">
         <v>9.8116238502</v>
-      </c>
-      <c r="E50" s="3">
-        <v>12.2185604292</v>
-      </c>
-      <c r="F50" s="3">
-        <v>10.4839102174</v>
       </c>
       <c r="G50" s="3"/>
       <c r="H50" s="3">
@@ -6512,10 +6512,10 @@
         </is>
       </c>
       <c r="C51" s="3">
-        <v>12.2185604292</v>
+        <v>13.9939353585</v>
       </c>
       <c r="D51" s="3">
-        <v>10.4839102174</v>
+        <v>12.0</v>
       </c>
       <c r="E51" s="3">
         <v>13.9155797828</v>
@@ -6545,10 +6545,10 @@
         </is>
       </c>
       <c r="C52" s="3">
-        <v>13.9155797828</v>
+        <v>14.7705439303</v>
       </c>
       <c r="D52" s="3">
-        <v>10.3899370543</v>
+        <v>10.6653787633</v>
       </c>
       <c r="E52" s="3">
         <v>14.1339424409</v>
@@ -6578,10 +6578,10 @@
         </is>
       </c>
       <c r="C53">
-        <v>14.1339424409</v>
+        <v>15.6500698835</v>
       </c>
       <c r="D53">
-        <v>10.2888438165</v>
+        <v>9.1419951257</v>
       </c>
       <c r="E53">
         <v>14.421771329</v>
@@ -6600,270 +6600,6 @@
       <c r="M53"/>
       <c r="N53"/>
       <c r="O53"/>
-    </row>
-    <row r="54">
-      <c r="A54">
-        <v>52</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>vor-51</t>
-        </is>
-      </c>
-      <c r="C54">
-        <v>14.421771329</v>
-      </c>
-      <c r="D54">
-        <v>9.3533122858</v>
-      </c>
-      <c r="E54">
-        <v>14.0108561039</v>
-      </c>
-      <c r="F54">
-        <v>8.724001641</v>
-      </c>
-      <c r="G54"/>
-      <c r="H54">
-        <v>35.0</v>
-      </c>
-      <c r="I54"/>
-      <c r="J54"/>
-      <c r="K54"/>
-      <c r="L54"/>
-      <c r="M54"/>
-      <c r="N54"/>
-      <c r="O54"/>
-    </row>
-    <row r="55">
-      <c r="A55">
-        <v>53</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>vor-52</t>
-        </is>
-      </c>
-      <c r="C55">
-        <v>14.3608123661</v>
-      </c>
-      <c r="D55">
-        <v>7.4155502673</v>
-      </c>
-      <c r="E55">
-        <v>14.0108561039</v>
-      </c>
-      <c r="F55">
-        <v>8.724001641</v>
-      </c>
-      <c r="G55"/>
-      <c r="H55">
-        <v>35.0</v>
-      </c>
-      <c r="I55"/>
-      <c r="J55"/>
-      <c r="K55"/>
-      <c r="L55"/>
-      <c r="M55"/>
-      <c r="N55"/>
-      <c r="O55"/>
-    </row>
-    <row r="56">
-      <c r="A56">
-        <v>54</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>vor-53</t>
-        </is>
-      </c>
-      <c r="C56">
-        <v>12.0382492411</v>
-      </c>
-      <c r="D56">
-        <v>7.5687085359</v>
-      </c>
-      <c r="E56">
-        <v>12.2927613852</v>
-      </c>
-      <c r="F56">
-        <v>8.8982603035</v>
-      </c>
-      <c r="G56"/>
-      <c r="H56">
-        <v>35.0</v>
-      </c>
-      <c r="I56"/>
-      <c r="J56"/>
-      <c r="K56"/>
-      <c r="L56"/>
-      <c r="M56"/>
-      <c r="N56"/>
-      <c r="O56"/>
-    </row>
-    <row r="57">
-      <c r="A57">
-        <v>55</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>vor-54</t>
-        </is>
-      </c>
-      <c r="C57">
-        <v>9.94722374</v>
-      </c>
-      <c r="D57">
-        <v>9.383846683</v>
-      </c>
-      <c r="E57">
-        <v>11.9559488087</v>
-      </c>
-      <c r="F57">
-        <v>9.8116238502</v>
-      </c>
-      <c r="G57"/>
-      <c r="H57">
-        <v>35.0</v>
-      </c>
-      <c r="I57"/>
-      <c r="J57"/>
-      <c r="K57"/>
-      <c r="L57"/>
-      <c r="M57"/>
-      <c r="N57"/>
-      <c r="O57"/>
-    </row>
-    <row r="58">
-      <c r="A58">
-        <v>56</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>vor-55</t>
-        </is>
-      </c>
-      <c r="C58">
-        <v>12.1925700451</v>
-      </c>
-      <c r="D58">
-        <v>10.582869313</v>
-      </c>
-      <c r="E58">
-        <v>12.2185604292</v>
-      </c>
-      <c r="F58">
-        <v>10.4839102174</v>
-      </c>
-      <c r="G58"/>
-      <c r="H58">
-        <v>35.0</v>
-      </c>
-      <c r="I58"/>
-      <c r="J58"/>
-      <c r="K58"/>
-      <c r="L58"/>
-      <c r="M58"/>
-      <c r="N58"/>
-      <c r="O58"/>
-    </row>
-    <row r="59">
-      <c r="A59">
-        <v>57</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>vor-56</t>
-        </is>
-      </c>
-      <c r="C59">
-        <v>13.9939353585</v>
-      </c>
-      <c r="D59">
-        <v>12.0</v>
-      </c>
-      <c r="E59">
-        <v>13.9155797828</v>
-      </c>
-      <c r="F59">
-        <v>10.3899370543</v>
-      </c>
-      <c r="G59"/>
-      <c r="H59">
-        <v>35.0</v>
-      </c>
-      <c r="I59"/>
-      <c r="J59"/>
-      <c r="K59"/>
-      <c r="L59"/>
-      <c r="M59"/>
-      <c r="N59"/>
-      <c r="O59"/>
-    </row>
-    <row r="60">
-      <c r="A60">
-        <v>58</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>vor-57</t>
-        </is>
-      </c>
-      <c r="C60">
-        <v>14.7705439303</v>
-      </c>
-      <c r="D60">
-        <v>10.6653787633</v>
-      </c>
-      <c r="E60">
-        <v>14.1339424409</v>
-      </c>
-      <c r="F60">
-        <v>10.2888438165</v>
-      </c>
-      <c r="G60"/>
-      <c r="H60">
-        <v>35.0</v>
-      </c>
-      <c r="I60"/>
-      <c r="J60"/>
-      <c r="K60"/>
-      <c r="L60"/>
-      <c r="M60"/>
-      <c r="N60"/>
-      <c r="O60"/>
-    </row>
-    <row r="61">
-      <c r="A61">
-        <v>59</v>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>vor-58</t>
-        </is>
-      </c>
-      <c r="C61">
-        <v>15.6500698835</v>
-      </c>
-      <c r="D61">
-        <v>9.1419951257</v>
-      </c>
-      <c r="E61">
-        <v>14.421771329</v>
-      </c>
-      <c r="F61">
-        <v>9.3533122858</v>
-      </c>
-      <c r="G61"/>
-      <c r="H61">
-        <v>35.0</v>
-      </c>
-      <c r="I61"/>
-      <c r="J61"/>
-      <c r="K61"/>
-      <c r="L61"/>
-      <c r="M61"/>
-      <c r="N61"/>
-      <c r="O61"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>